<commit_message>
data: reconcile Demo workbook values and recording reward timing
</commit_message>
<xml_diff>
--- a/luban-excels/xlsx/Items.xlsx
+++ b/luban-excels/xlsx/Items.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="12851" tabRatio="812" activeTab="5"/>
+    <workbookView windowWidth="29868" windowHeight="13451" tabRatio="812" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Item" sheetId="1" r:id="rId1"/>
@@ -22642,7 +22642,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="49" operator="containsText" id="{cc9b94e1-10b8-4681-ba51-208005966965}">
+          <x14:cfRule type="containsText" priority="49" operator="containsText" id="{1f2f65b8-84f7-4abb-b4ab-e76391d86592}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L62)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22656,7 +22656,7 @@
           <xm:sqref>L62</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="44" operator="containsText" id="{11c639cb-7d41-472a-bf30-e6288d2e1a5c}">
+          <x14:cfRule type="containsText" priority="44" operator="containsText" id="{752aede5-0836-471a-8f75-7c1f7c6fd7f9}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L63)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22670,7 +22670,7 @@
           <xm:sqref>L63</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="29" operator="containsText" id="{77a7fb3f-2135-4e35-b1a1-a7eba2ecc045}">
+          <x14:cfRule type="containsText" priority="29" operator="containsText" id="{8a3dec2d-f6fe-4512-9623-33bd0a254a9a}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L64)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22684,7 +22684,7 @@
           <xm:sqref>L64</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="39" operator="containsText" id="{1710f7a4-9cea-4018-987a-06ffd3718110}">
+          <x14:cfRule type="containsText" priority="39" operator="containsText" id="{19ad3260-f832-4893-a669-0c1479b0ef5f}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L70)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22698,7 +22698,7 @@
           <xm:sqref>L70</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="34" operator="containsText" id="{ce25aff1-1d39-42da-84eb-6e911686a559}">
+          <x14:cfRule type="containsText" priority="34" operator="containsText" id="{844be943-525f-4fe5-95fc-3a6f243a674e}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L71)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22712,7 +22712,7 @@
           <xm:sqref>L71</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="24" operator="containsText" id="{05bdb030-492c-4b1e-b55e-df641a7bc0ce}">
+          <x14:cfRule type="containsText" priority="24" operator="containsText" id="{a4a4377e-39b6-499b-8679-48178d0f0594}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L72)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22726,7 +22726,7 @@
           <xm:sqref>L72</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="9" operator="containsText" id="{7460289d-0e01-47bf-9fc4-1ea086902fc0}">
+          <x14:cfRule type="containsText" priority="9" operator="containsText" id="{59456909-59a9-4470-a7cd-2aaf30496b60}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L13)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22740,7 +22740,7 @@
           <xm:sqref>L13:L16</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{7b78b252-a15d-48c9-97a9-61e68c0afaac}">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{ede9442d-536c-4e57-825a-016dc13975b5}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L17)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -22754,7 +22754,7 @@
           <xm:sqref>L17:L20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="54" operator="containsText" id="{14c66c72-7b4b-4a84-93e3-1e760d2416cd}">
+          <x14:cfRule type="containsText" priority="54" operator="containsText" id="{52aeb0ed-bb8b-4f17-ac77-e31ad6fde35d}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,L1)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>
@@ -24748,7 +24748,7 @@
         <v>3</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L5" t="s">
         <v>827</v>
@@ -24789,7 +24789,7 @@
         <v>3</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L6" t="s">
         <v>827</v>
@@ -24830,7 +24830,7 @@
         <v>3</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L7" t="s">
         <v>827</v>
@@ -24862,7 +24862,7 @@
         <v>825</v>
       </c>
       <c r="H8">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="I8" t="s">
         <v>826</v>
@@ -24871,7 +24871,7 @@
         <v>3</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L8" t="s">
         <v>827</v>
@@ -24903,7 +24903,7 @@
         <v>825</v>
       </c>
       <c r="H9">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="I9" t="s">
         <v>826</v>
@@ -24912,7 +24912,7 @@
         <v>3</v>
       </c>
       <c r="K9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L9" t="s">
         <v>827</v>
@@ -24953,7 +24953,7 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L10" t="s">
         <v>827</v>
@@ -24991,7 +24991,7 @@
         <v>3</v>
       </c>
       <c r="K11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L11" t="s">
         <v>841</v>
@@ -25032,7 +25032,7 @@
         <v>3</v>
       </c>
       <c r="K12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L12" t="s">
         <v>827</v>
@@ -26271,7 +26271,7 @@
         <v>0</v>
       </c>
       <c r="U20">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V20">
         <v>0</v>
@@ -26337,7 +26337,7 @@
         <v>0</v>
       </c>
       <c r="U21">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V21">
         <v>0</v>
@@ -26403,7 +26403,7 @@
         <v>0</v>
       </c>
       <c r="U22">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V22">
         <v>0</v>
@@ -26469,7 +26469,7 @@
         <v>0</v>
       </c>
       <c r="U23">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V23">
         <v>0</v>
@@ -26535,7 +26535,7 @@
         <v>0</v>
       </c>
       <c r="U24">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V24">
         <v>0</v>
@@ -26601,7 +26601,7 @@
         <v>0</v>
       </c>
       <c r="U25">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V25">
         <v>0</v>
@@ -26667,7 +26667,7 @@
         <v>0</v>
       </c>
       <c r="U26">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V26">
         <v>0</v>
@@ -26733,7 +26733,7 @@
         <v>0</v>
       </c>
       <c r="U27">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V27">
         <v>0</v>
@@ -26799,7 +26799,7 @@
         <v>0</v>
       </c>
       <c r="U28">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V28">
         <v>0</v>
@@ -26865,7 +26865,7 @@
         <v>0</v>
       </c>
       <c r="U29">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V29">
         <v>0</v>
@@ -26931,7 +26931,7 @@
         <v>0</v>
       </c>
       <c r="U30">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V30">
         <v>0</v>
@@ -26997,7 +26997,7 @@
         <v>0</v>
       </c>
       <c r="U31">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V31">
         <v>0</v>
@@ -27063,7 +27063,7 @@
         <v>0</v>
       </c>
       <c r="U32">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V32">
         <v>0</v>
@@ -27129,7 +27129,7 @@
         <v>0</v>
       </c>
       <c r="U33">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V33">
         <v>0</v>
@@ -27195,7 +27195,7 @@
         <v>0</v>
       </c>
       <c r="U34">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="V34">
         <v>0</v>

</xml_diff>